<commit_message>
Add SCF equivalent control mapping for SIMM 5310-B (Individual Access to Personal Information)
Maps each requirement of the SIMM 5310-B standard (response to requests
for information, response timeframes, time limits for record access,
access denial/recourse, permitting an agent access, and protecting
other individuals' information in a disclosure) to the corresponding
Secure Controls Framework Data Privacy (PRI) controls, following the
same FDE-to-SCF STRM format used elsewhere in the workbook.
</commit_message>
<xml_diff>
--- a/SAMSCF-SAM5300-Mapping.xlsx
+++ b/SAMSCF-SAM5300-Mapping.xlsx
@@ -1558,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1719"/>
+  <dimension ref="A1:K1728"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="22.3671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="22.3671875" customWidth="1" style="1" min="1" max="2"/>
@@ -58516,6 +58516,491 @@
       <c r="K1719" s="32" t="inlineStr">
         <is>
           <t>Added on review: DCH-09.3 mandates sanitization of Personal Data (PD) specifically -- a narrower instance of the SAM provision's broader requirement to sanitize all digital/non-digital media prior to disposal or reuse, regardless of data type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P01</t>
+        </is>
+      </c>
+      <c r="B1720" s="32" t="inlineStr">
+        <is>
+          <t>INTRODUCTION</t>
+        </is>
+      </c>
+      <c r="C1720" s="32" t="inlineStr">
+        <is>
+          <t>This standard provides requirements to information asset custodians and state entity personnel on the parameters under which individuals shall be provided access to personal information that has been collected by agencies.</t>
+        </is>
+      </c>
+      <c r="D1720" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1720" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy Program</t>
+        </is>
+      </c>
+      <c r="F1720" s="23" t="inlineStr">
+        <is>
+          <t>PRI-01</t>
+        </is>
+      </c>
+      <c r="G1720" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to facilitate the implementation and operation of data protection controls throughout the data lifecycle to ensure all forms of Personal Data (PD) are processed lawfully, fairly and transparently.</t>
+        </is>
+      </c>
+      <c r="H1720" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1720" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1720" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1720" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. The FDE's overarching mandate to govern the parameters under which individuals are provided access to personal information collected by agencies addresses the same subject matter as PRI-01's data privacy program, but PRI-01 covers the full data lifecycle while the FDE is scoped specifically to individual-access requirements, so the controls intersect rather than align exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P02</t>
+        </is>
+      </c>
+      <c r="B1721" s="32" t="inlineStr">
+        <is>
+          <t>RESPONSE TO REQUESTS FOR INFORMATION</t>
+        </is>
+      </c>
+      <c r="C1721" s="32" t="inlineStr">
+        <is>
+          <t>If an individual requests information as to whether or not a state entity maintains a record of personal information about that individual, the state entity shall include in the response, at least, the state entity's Privacy Policy Statement and the state entity's relevant Privacy Notice on Collection. Both of these documents shall meet or exceed the requirements contained in the Privacy Statement and Notices Standard (SIMM 5310-A).</t>
+        </is>
+      </c>
+      <c r="D1721" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1721" s="23" t="inlineStr">
+        <is>
+          <t>Data Subject Empowerment</t>
+        </is>
+      </c>
+      <c r="F1721" s="23" t="inlineStr">
+        <is>
+          <t>PRI-06</t>
+        </is>
+      </c>
+      <c r="G1721" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provide authenticated data subjects the ability to:
+(1) Access their Personal Data (PD) that is being processed, stored and shared, except where the burden, risk or expense of providing access would be disproportionate to the benefit offered to the data subject through granting access;
+(2) Obtain answers on the specifics of how their PD is collected, received, processed, stored, transmitted, shared, updated and/or disposed; 
+(3) Obtain the source(s) of their PD; 
+(4) Obtain the categories of their PD being collected, received, processed, stored and shared; 
+(5) Request correction to their PD due to inaccuracies;
+(6) Request erasure of their PD; and
+(7) Restrict the further collecting, receiving, processing, storing, transmitting, updated and/or sharing of their PD.</t>
+        </is>
+      </c>
+      <c r="H1721" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1721" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1721" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1721" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Responding to an individual's request to confirm whether the state entity maintains a record of PD about them is a specific instance of PRI-06's broader right for authenticated data subjects to obtain answers on the specifics of how their PD is collected and processed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="32" t="n"/>
+      <c r="B1722" s="32" t="n"/>
+      <c r="C1722" s="32" t="n"/>
+      <c r="D1722" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1722" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy Notice</t>
+        </is>
+      </c>
+      <c r="F1722" s="23" t="inlineStr">
+        <is>
+          <t>PRI-02</t>
+        </is>
+      </c>
+      <c r="G1722" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to: (1) Make data privacy notice(s) available to individuals upon first interacting with an organization and subsequently as necessary; (2) Ensure that data privacy notices are clear and easy-to-understand, expressing relevant information about how Personal Data (PD) is collected, received, processed, stored, transmitted, shared, updated and/or disposed; (3) Contain all necessary notice-related criteria required by applicable statutory, regulatory and contractual obligations; (4) Define the scope of PD processing activities, including the geographic locations and third-party recipients that process the PD within the scope of the data privacy notice; (5) Periodically, review and update the content of the privacy notice, as necessary; and (6) Retain prior versions of the privacy notice, in accordance with data retention requirements.</t>
+        </is>
+      </c>
+      <c r="H1722" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1722" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1722" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1722" s="32" t="inlineStr">
+        <is>
+          <t>The requirement that the Privacy Policy Statement and Privacy Notice on Collection provided in response to an individual's inquiry meet or exceed the Privacy Statement and Notices Standard (SIMM 5310-A) overlaps with PRI-02's mandate that data privacy notices be clear and contain all necessary notice-related criteria; PRI-02 governs notice content and availability generally, while the FDE ties that content standard specifically to responding to individual requests, so the controls intersect rather than align exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P03</t>
+        </is>
+      </c>
+      <c r="B1723" s="32" t="inlineStr">
+        <is>
+          <t>TIME FRAME FOR RESPONSE</t>
+        </is>
+      </c>
+      <c r="C1723" s="32" t="inlineStr">
+        <is>
+          <t>The trustee shall inform the individual requesting information of the timeframe in which they can expect a response from the state entity. The state entity shall respond to requests for information within 30 days.</t>
+        </is>
+      </c>
+      <c r="D1723" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1723" s="23" t="inlineStr">
+        <is>
+          <t>Data Subject Feedback Management</t>
+        </is>
+      </c>
+      <c r="F1723" s="23" t="inlineStr">
+        <is>
+          <t>PRI-06.4</t>
+        </is>
+      </c>
+      <c r="G1723" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to maintain a process to efficiently and effectively respond to requests, complaints, concerns and/or questions from authenticated data subjects about Personal Data (PD) the organization collects, receives, processes, stores, transmits, shares, updates and/or disposes.</t>
+        </is>
+      </c>
+      <c r="H1723" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1723" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1723" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1723" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Informing individuals of, and meeting, a defined 30-day timeframe for responding to information requests is part of the process PRI-06.4 requires for responding efficiently and effectively to data subject requests; PRI-06.4 does not itself mandate a specific timeframe or advance notice of it, so the controls intersect rather than align exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P04</t>
+        </is>
+      </c>
+      <c r="B1724" s="32" t="inlineStr">
+        <is>
+          <t>TIME LIMITS</t>
+        </is>
+      </c>
+      <c r="C1724" s="32" t="inlineStr">
+        <is>
+          <t>Upon request and proper identification, individuals shall be provided access to his or her record within 30 days of the state entity's receipt of the request if the record is active, and within 60 days of the state entity's receipt of the request for records that are in multiple locations, or which are inactive and in central storage. All access requests pertaining to records containing personal information are subject to limitations as described in the Information Practices Act of 1977 as well as the SAM section 5365, Privacy Policy.</t>
+        </is>
+      </c>
+      <c r="D1724" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1724" s="23" t="inlineStr">
+        <is>
+          <t>Data Subject Empowerment</t>
+        </is>
+      </c>
+      <c r="F1724" s="23" t="inlineStr">
+        <is>
+          <t>PRI-06</t>
+        </is>
+      </c>
+      <c r="G1724" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provide authenticated data subjects the ability to:
+(1) Access their Personal Data (PD) that is being processed, stored and shared, except where the burden, risk or expense of providing access would be disproportionate to the benefit offered to the data subject through granting access;
+(2) Obtain answers on the specifics of how their PD is collected, received, processed, stored, transmitted, shared, updated and/or disposed; 
+(3) Obtain the source(s) of their PD; 
+(4) Obtain the categories of their PD being collected, received, processed, stored and shared; 
+(5) Request correction to their PD due to inaccuracies;
+(6) Request erasure of their PD; and
+(7) Restrict the further collecting, receiving, processing, storing, transmitting, updated and/or sharing of their PD.</t>
+        </is>
+      </c>
+      <c r="H1724" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1724" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1724" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1724" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Providing individuals access to their own records upon request and proper identification is the core activity PRI-06 addresses by granting authenticated data subjects the ability to access their PD; PRI-06 does not specify the 30/60-day timeframes or the statutory limitations the FDE imposes, so the relationship is an intersection rather than a subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P05</t>
+        </is>
+      </c>
+      <c r="B1725" s="32" t="inlineStr">
+        <is>
+          <t>ACCESS DENIAL</t>
+        </is>
+      </c>
+      <c r="C1725" s="32" t="inlineStr">
+        <is>
+          <t>If a state entity denies an individual access to his or her records of personal information, the individual shall be provided with an explanation of the reason for denial. The individual shall be informed of the state entity's method of recourse if the individual disputes the decision to deny access, including an explanation of the right to bring a civil action, as per Civil Code section 1798.45.</t>
+        </is>
+      </c>
+      <c r="D1725" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1725" s="23" t="inlineStr">
+        <is>
+          <t>Justification To Reject Disclosure Requests</t>
+        </is>
+      </c>
+      <c r="F1725" s="23" t="inlineStr">
+        <is>
+          <t>PRI-07.5</t>
+        </is>
+      </c>
+      <c r="G1725" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to document justifiable reasons for rejecting a data subject's access request for disclosure when the request is: (1) Harassing; (2) Repetitive; (3) Fraudulent; (4) Unjustified; and/or (5) Unlawful.</t>
+        </is>
+      </c>
+      <c r="H1725" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1725" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1725" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1725" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Providing an individual with an explanation of the reason a records-access request was denied is a specific instance of PRI-07.5's broader requirement to document justifiable reasons for rejecting a data subject's access/disclosure request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="32" t="n"/>
+      <c r="B1726" s="32" t="n"/>
+      <c r="C1726" s="32" t="n"/>
+      <c r="D1726" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1726" s="23" t="inlineStr">
+        <is>
+          <t>Appeal Adverse Decision</t>
+        </is>
+      </c>
+      <c r="F1726" s="23" t="inlineStr">
+        <is>
+          <t>PRI-06.3</t>
+        </is>
+      </c>
+      <c r="G1726" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to maintain a process for data subjects to appeal an adverse decision.</t>
+        </is>
+      </c>
+      <c r="H1726" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1726" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1726" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1726" s="32" t="inlineStr">
+        <is>
+          <t>Informing the individual of the state entity's method of recourse, including the right to bring a civil action under Civil Code section 1798.45, if they dispute a denial overlaps with PRI-06.3's mandate to maintain a process for data subjects to appeal an adverse decision; PRI-06.3 does not address the statutory civil-action right the FDE cites, so the controls intersect rather than align exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P06</t>
+        </is>
+      </c>
+      <c r="B1727" s="32" t="inlineStr">
+        <is>
+          <t>PERMITTING OTHER INDIVIDUALS ACCESS</t>
+        </is>
+      </c>
+      <c r="C1727" s="32" t="inlineStr">
+        <is>
+          <t>Upon request, an individual may appoint an agent of his or her choosing to access any or all records of personal information and to have an exact copy made of all or any portion of the record within 15 days of the inspection. A state entity may require the individual to provide a written statement authorizing disclosure of the individual's record to the agent.</t>
+        </is>
+      </c>
+      <c r="D1727" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1727" s="23" t="inlineStr">
+        <is>
+          <t>Authorized Agent</t>
+        </is>
+      </c>
+      <c r="F1727" s="23" t="inlineStr">
+        <is>
+          <t>PRI-03.6</t>
+        </is>
+      </c>
+      <c r="G1727" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to allow data subjects to authorize another person or entity (e.g., authorized agent, proxy, etc.), acting on the data subject's behalf, to make Personal Data (PD) processing decisions.</t>
+        </is>
+      </c>
+      <c r="H1727" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1727" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1727" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1727" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Allowing an individual to appoint an agent to access and obtain copies of their records, optionally supported by a written authorization statement, is a specific instance of PRI-03.6's broader mechanism allowing data subjects to authorize another person or entity to act on their behalf regarding their PD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="32" t="inlineStr">
+        <is>
+          <t>5310-B P07</t>
+        </is>
+      </c>
+      <c r="B1728" s="32" t="inlineStr">
+        <is>
+          <t>INFORMATION RELATING TO OTHER INDIVIDUALS</t>
+        </is>
+      </c>
+      <c r="C1728" s="32" t="inlineStr">
+        <is>
+          <t>In disclosing personal information contained in a record to one individual, no personal information relating to another second individual shall be contained in the record. To comply with this section, all personal information concerning the second individual shall be deleted from the copy provided to the first, or otherwise removed from the disclosure.</t>
+        </is>
+      </c>
+      <c r="D1728" s="23" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+      <c r="E1728" s="23" t="inlineStr">
+        <is>
+          <t>Data Anonymization</t>
+        </is>
+      </c>
+      <c r="F1728" s="23" t="inlineStr">
+        <is>
+          <t>PRI-05.3</t>
+        </is>
+      </c>
+      <c r="G1728" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to mask sensitive and/or regulated data through data anonymization, pseudonymization, redaction and/or de-identification.</t>
+        </is>
+      </c>
+      <c r="H1728" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1728" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1728" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1728" s="32" t="inlineStr">
+        <is>
+          <t>Confirmed. Requiring that a second individual's personal information be deleted or otherwise removed before disclosing a record to the first individual is a specific application of PRI-05.3's broader mandate to mask sensitive data through anonymization, pseudonymization, redaction and/or de-identification.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Decompose SIMM 5315-A Email Threat Protection Standard into atomic controls and map to SCF v2026.2
Break SIMM 5315-A (Protection, Detection, Investigative Support,
Containment, Remediation, and above-minimum capabilities) into 38
granular "Mechanisms exist to..." atomic control statements, then STRM
map each to SCF v2026.2 (36 matched across 48 mapping rows, 2 No Match).

- Add SIMM-5315-A-ETP-SCF-Mapping.xlsx: standalone crosswalk for the
  standard, same template structure as the SAM 5300 mapping.
- Update SAMSCF-SAM5300-Mapping.xlsx: fold the same 38 FDEs in as
  additional rows (FDE # prefixed "5315-A"), providing the detail
  behind SAM 5315's Implementation Controls citation of SIMM 5315-A.
  All 224 existing SAM 5300 FDE mappings are untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019X35PyKa6oSXdsYgyQ1vJS
</commit_message>
<xml_diff>
--- a/SAMSCF-SAM5300-Mapping.xlsx
+++ b/SAMSCF-SAM5300-Mapping.xlsx
@@ -1558,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1719"/>
+  <dimension ref="A1:K1750"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="22.3671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="22.3671875" customWidth="1" style="1" min="1" max="2"/>
@@ -2019,6 +2019,21 @@
       </c>
     </row>
     <row r="11" ht="130.5" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5315-A PROT-10b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to require entity ISO approval for exceptions to the default prohibition on external auto-forwarding.</t>
+        </is>
+      </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
           <t>Security, Compliance &amp; Resilience Governance</t>
@@ -2039,8 +2054,24 @@
           <t>Mechanisms exist to prohibit exceptions to standards, except when the exception has been formally assessed for risk impact, approved and recorded.</t>
         </is>
       </c>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="12" t="n"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>GOV-02.1's requirement that exceptions to standards be formally risk-assessed, approved and recorded matches almost exactly the FDE's requirement that ISO approval govern any exception to the default auto-forwarding prohibition.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="130.5" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -16189,6 +16220,21 @@
       </c>
     </row>
     <row r="472" ht="77.40000000000001" customHeight="1">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>5315-A INV-00</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to search the entire email store for specific emails or indicators and provide results to administrators for further action.</t>
+        </is>
+      </c>
       <c r="D472" s="23" t="inlineStr">
         <is>
           <t>Continuous Monitoring</t>
@@ -16207,6 +16253,24 @@
       <c r="G472" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to utilize a Security Incident Event Manager (SIEM), or similar automated tool, to support the centralized collection of security-related event logs.</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J472" t="n">
+        <v>5</v>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>Centralized collection of security event logs (MON-02) provides a similar searchable-record capability, though it is framed around security event logs generally rather than the full email store.</t>
         </is>
       </c>
     </row>
@@ -20348,6 +20412,21 @@
       </c>
     </row>
     <row r="605" ht="64.5" customHeight="1">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>5315-A INV-02</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to transmit pertinent cyber threat information, consistent with NIST SP 800-150, to the California Department of Technology.</t>
+        </is>
+      </c>
       <c r="D605" s="23" t="inlineStr">
         <is>
           <t>Data Classification &amp; Handling</t>
@@ -20366,6 +20445,24 @@
       <c r="G605" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to utilize a process to assist users in making information sharing decisions to ensure data is appropriately protected.</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J605" t="n">
+        <v>5</v>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>DCH-14's process to guide appropriate information-sharing decisions overlaps with sharing threat information externally, though DCH-14 is general-purpose rather than threat-intelligence-specific.</t>
         </is>
       </c>
     </row>
@@ -20623,6 +20720,21 @@
       </c>
     </row>
     <row r="616" ht="116.1" customHeight="1">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>5315-A PROT-08</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict email operations, mail stores, and administrative activity to reside within the continental United States.</t>
+        </is>
+      </c>
       <c r="D616" s="23" t="inlineStr">
         <is>
           <t>Data Classification &amp; Handling</t>
@@ -20641,6 +20753,24 @@
       <c r="G616" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to inventory, document and maintain data flows for data that is resident (permanently or temporarily) within a service's geographically distributed applications (physical and virtual), infrastructure, systems components and/or shared with other third-parties.</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J616" t="n">
+        <v>5</v>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>DCH-19 requires inventorying/documenting the geographic location of distributed data generally; this FDE imposes a specific US-only residency constraint on email operations, a narrower and more prescriptive rule than DCH-19's documentation mandate.</t>
         </is>
       </c>
     </row>
@@ -21184,6 +21314,21 @@
       </c>
     </row>
     <row r="637" ht="129" customHeight="1">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>5315-A PROT-08</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict email operations, mail stores, and administrative activity to reside within the continental United States.</t>
+        </is>
+      </c>
       <c r="D637" s="23" t="inlineStr">
         <is>
           <t>Data Classification &amp; Handling</t>
@@ -21202,6 +21347,24 @@
       <c r="G637" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to constrain the impact of "digital sovereignty laws," that require localized data within the host country, where data and processes may be subjected to arbitrary enforcement actions that potentially violate other applicable statutory, regulatory and/or contractual obligations.</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J637" t="n">
+        <v>5</v>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>DCH-26 addresses constraining impacts of foreign data-localization/sovereignty laws; this FDE is a state-imposed US-residency requirement rather than a response to a foreign sovereignty law, so overlap is conceptual (geographic data control) rather than mechanism-identical.</t>
         </is>
       </c>
     </row>
@@ -22675,6 +22838,21 @@
       </c>
     </row>
     <row r="685" ht="90.3" customHeight="1">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>5315-A REM-01</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Remediation Capabilities</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement custom filtering of incoming email to screen for previously detected malicious emails.</t>
+        </is>
+      </c>
       <c r="D685" s="23" t="inlineStr">
         <is>
           <t>Endpoint Security</t>
@@ -22693,6 +22871,24 @@
       <c r="G685" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to automatically update anti-phishing and spam protection technologies when new releases are available in accordance with configuration and change management practices.</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J685" t="n">
+        <v>5</v>
+      </c>
+      <c r="K685" t="inlineStr">
+        <is>
+          <t>Automatic updates to spam/phishing protections when new detections occur overlaps conceptually with continuously filtering for previously detected malicious emails, though the specific 'custom filter based on prior detections' mechanism isn't directly addressed.</t>
         </is>
       </c>
     </row>
@@ -26616,6 +26812,21 @@
       </c>
     </row>
     <row r="818" ht="51.6" customHeight="1">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>5315-A OPT-02</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Above-Minimum / Optional Capabilities</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict who may send to group/distribution email lists, preventing external entities from using an entity's internal distribution lists.</t>
+        </is>
+      </c>
       <c r="D818" s="23" t="inlineStr">
         <is>
           <t>Identification &amp; Authentication</t>
@@ -26634,6 +26845,24 @@
       <c r="G818" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to authorize the use of shared/group accounts only under certain organization-defined conditions.</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J818" t="n">
+        <v>5</v>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>Restricting who may send to group/distribution email lists overlaps with IAC-15.5's authorization conditions for shared/group accounts, though IAC-15.5 is framed around account usage generally rather than distribution-list send permissions specifically.</t>
         </is>
       </c>
     </row>
@@ -28814,6 +29043,21 @@
       </c>
     </row>
     <row r="886" ht="77.40000000000001" customHeight="1">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>5315-A INV-00</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to search the entire email store for specific emails or indicators and provide results to administrators for further action.</t>
+        </is>
+      </c>
       <c r="D886" s="23" t="inlineStr">
         <is>
           <t>Incident Response</t>
@@ -28832,6 +29076,24 @@
       <c r="G886" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to perform digital forensics and maintain the integrity of the chain of custody, in accordance with applicable laws, regulations and industry-recognized secure practices.</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J886" t="n">
+        <v>5</v>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>Searching the email store for specific emails/indicators supports digital forensics and investigations, overlapping with IRO-08's chain-of-custody/forensics mandate, though IRO-08 is broader (all forensics) and not specific to email search capability.</t>
         </is>
       </c>
     </row>
@@ -29628,6 +29890,21 @@
       </c>
     </row>
     <row r="909" ht="64.5" customHeight="1">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>5315-A DET-02</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to screen email attachments using malware analysis, sandboxing, and machine learning to block malicious attachments, including zero-day threats, prior to delivery.</t>
+        </is>
+      </c>
       <c r="D909" s="23" t="inlineStr">
         <is>
           <t>Incident Response</t>
@@ -29646,6 +29923,24 @@
       <c r="G909" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to utilize a detonation chamber capability to detect and/or block potentially-malicious files and email attachments.</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J909" t="n">
+        <v>10</v>
+      </c>
+      <c r="K909" t="inlineStr">
+        <is>
+          <t>Screening attachments via sandbox/malware analysis to block malicious attachments including zero-day is a specific instance of IRO-15's mandate to use detonation chambers to detect/block malicious files and email attachments.</t>
         </is>
       </c>
     </row>
@@ -32535,6 +32830,21 @@
       </c>
     </row>
     <row r="1020" ht="129" customHeight="1">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>5315-A PROT-01b</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement SPF (Sender Policy Framework) to validate authorized senders for a domain.</t>
+        </is>
+      </c>
       <c r="D1020" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -32553,6 +32863,24 @@
       <c r="G1020" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to validate the legitimacy of email communications through configuring a Domain Naming Service (DNS) Sender Policy Framework (SPF) record to specify the IP addresses and/or hostnames that are authorized to send email from the specified domain.</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1020" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>Both require configuring an SPF DNS record specifying authorized senders for the domain; scope is essentially identical.</t>
         </is>
       </c>
     </row>
@@ -33441,6 +33769,21 @@
       </c>
     </row>
     <row r="1043" ht="64.5" customHeight="1">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>5315-A PROT-09</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to apply data loss prevention (DLP) to outbound email to detect and prevent unauthorized transmission of confidential, sensitive, or personal information.</t>
+        </is>
+      </c>
       <c r="D1043" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33461,8 +33804,41 @@
           <t>Automated mechanisms exist to implement Data Loss Prevention (DLP) to protect sensitive information as it is stored, transmitted and processed.</t>
         </is>
       </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1043" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>Both require automated data loss prevention on outbound information to detect/prevent unauthorized transmission of sensitive data; scope is essentially identical.</t>
+        </is>
+      </c>
     </row>
     <row r="1044" ht="103.2" customHeight="1">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>5315-A PROT-12</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to apply DNS filtering to email-related traffic.</t>
+        </is>
+      </c>
       <c r="D1044" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33481,6 +33857,24 @@
       <c r="G1044" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to force Internet-bound network traffic through a proxy device (e.g., Policy Enforcement Point (PEP)) for URL content filtering and DNS filtering to limit a user's ability to connect to dangerous or prohibited Internet sites.</t>
+        </is>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1044" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>Applying DNS filtering to email-related traffic is a specific instance of NET-18's broader DNS &amp; content filtering mandate.</t>
         </is>
       </c>
     </row>
@@ -33705,6 +34099,21 @@
       </c>
     </row>
     <row r="1055" ht="64.5" customHeight="1">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>5315-A DET-01</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to screen inbound email for spam, phishing, and malicious intent using heuristics and machine learning, quarantining likely malicious or phishing emails.</t>
+        </is>
+      </c>
       <c r="D1055" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33725,8 +34134,41 @@
           <t>Mechanisms exist to implement an email filtering security service to detect malicious attachments in emails and prevent users from accessing them.</t>
         </is>
       </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1055" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1055" t="inlineStr">
+        <is>
+          <t>NET-20's email filtering service to detect malicious content overlaps with spam/phishing screening but is framed around attachments specifically rather than the full spam/phishing/malicious-intent screening scope.</t>
+        </is>
+      </c>
     </row>
     <row r="1056" ht="51.6" customHeight="1">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>5315-A PROT-05</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement domain reputation-based protections for email.</t>
+        </is>
+      </c>
       <c r="D1056" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33745,6 +34187,24 @@
       <c r="G1056" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to monitor the organization's email domain’s reputation and protect the email domain’s reputation.</t>
+        </is>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1056" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>Both require monitoring and protecting email domain reputation; scope is essentially identical.</t>
         </is>
       </c>
     </row>
@@ -33771,6 +34231,21 @@
       </c>
     </row>
     <row r="1058" ht="103.2" customHeight="1">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>5315-A PROT-04</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to detect email spoofing of both internal and external domains.</t>
+        </is>
+      </c>
       <c r="D1058" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33791,8 +34266,41 @@
           <t>Mechanisms exist to utilize an authenticated received chain that allows for an intermediary to sign its own authentication of the original email, allowing downstream entities to accept the intermediary’s authentication even if the email was changed.</t>
         </is>
       </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1058" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>ARC supports validating an email's authentication chain across intermediaries, which helps detect certain spoofing/tampering scenarios, but is narrower in mechanism than general spoofing detection.</t>
+        </is>
+      </c>
     </row>
     <row r="1059" ht="90.3" customHeight="1">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>5315-A PROT-01a</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement the DMARC authentication and policy enforcement protocol for email domains.</t>
+        </is>
+      </c>
       <c r="D1059" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33813,8 +34321,41 @@
           <t>Mechanisms exist to implement domain signature verification protections that authenticate incoming email according to the Domain-based Message Authentication Reporting and Conformance (DMARC).</t>
         </is>
       </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1059" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1059" t="inlineStr">
+        <is>
+          <t>Both require implementing DMARC as the domain signature verification/authentication protocol for incoming email; scope and mechanism are essentially identical.</t>
+        </is>
+      </c>
     </row>
     <row r="1060" ht="116.1" customHeight="1">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>5315-A PROT-01c</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement DKIM (DomainKeys Identified Mail) to cryptographically validate email origin and integrity.</t>
+        </is>
+      </c>
       <c r="D1060" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33835,8 +34376,41 @@
           <t>Mechanisms exist to enable users to digitally sign their emails, allowing external parties to authenticate the email’s sender and its contents according to the Domain-based Message Authentication Reporting and Conformance (DMARC) email authentication protocol.</t>
         </is>
       </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1060" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1060" t="inlineStr">
+        <is>
+          <t>DKIM and NET-20.5's user-level digital signing both cryptographically authenticate email origin/integrity, but DKIM is a domain-level signing standard while NET-20.5 is framed around individual users digitally signing their own emails -- related mechanisms, not identical scope.</t>
+        </is>
+      </c>
     </row>
     <row r="1061" ht="51.6" customHeight="1">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>5315-A PROT-06a</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provide on-demand email encryption for messages containing confidential, sensitive, or personal information when required by policy or law.</t>
+        </is>
+      </c>
       <c r="D1061" s="23" t="inlineStr">
         <is>
           <t>Network Security</t>
@@ -33855,6 +34429,24 @@
       <c r="G1061" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to enable the encryption of outgoing emails using organization-approved cryptographic means.</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1061" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1061" t="inlineStr">
+        <is>
+          <t>On-demand user-triggered encryption of sensitive email is a specific instance of NET-20.6's broader mandate to enable encryption of outgoing email.</t>
         </is>
       </c>
     </row>
@@ -46709,6 +47301,21 @@
       </c>
     </row>
     <row r="1475" ht="129" customHeight="1">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>5315-A PROT-03</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to incorporate vendor-provided threat intelligence into email protection capabilities.</t>
+        </is>
+      </c>
       <c r="D1475" s="23" t="inlineStr">
         <is>
           <t>Threat Management</t>
@@ -46727,6 +47334,24 @@
       <c r="G1475" s="24" t="inlineStr">
         <is>
           <t>Mechanisms exist to implement a threat intelligence program that includes a cross-organization information-sharing capability that can influence the development of the system and security architectures, selection of security solutions, monitoring, threat hunting, response and recovery activities.</t>
+        </is>
+      </c>
+      <c r="H1475" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1475" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1475" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1475" t="inlineStr">
+        <is>
+          <t>Vendor threat intelligence feeding email protections overlaps with THR-01's broader cross-organizational threat intelligence program, though THR-01 is much wider in scope than this single email use case.</t>
         </is>
       </c>
     </row>
@@ -58516,6 +59141,1695 @@
       <c r="K1719" s="32" t="inlineStr">
         <is>
           <t>Added on review: DCH-09.3 mandates sanitization of Personal Data (PD) specifically -- a narrower instance of the SAM provision's broader requirement to sanitize all digital/non-digital media prior to disposal or reuse, regardless of data type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="32" t="inlineStr">
+        <is>
+          <t>5315-A GOV-01</t>
+        </is>
+      </c>
+      <c r="B1720" s="32" t="inlineStr">
+        <is>
+          <t>Introduction / Scope</t>
+        </is>
+      </c>
+      <c r="C1720" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to ensure email services include the minimum email threat protections defined by this standard.</t>
+        </is>
+      </c>
+      <c r="D1720" s="23" t="inlineStr">
+        <is>
+          <t>Security, Compliance &amp; Resilience Governance</t>
+        </is>
+      </c>
+      <c r="E1720" s="23" t="inlineStr">
+        <is>
+          <t>Security, Compliance &amp; Resilience Program (SCRP)</t>
+        </is>
+      </c>
+      <c r="F1720" s="23" t="inlineStr">
+        <is>
+          <t>GOV-01</t>
+        </is>
+      </c>
+      <c r="G1720" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to facilitate the implementation of security, compliance and resilience governance controls.</t>
+        </is>
+      </c>
+      <c r="H1720" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1720" s="33" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1720" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1720" s="32" t="inlineStr">
+        <is>
+          <t>Ensuring email services include this standard's minimum protections is the state-specific instantiation of GOV-01's broader mandate to facilitate implementation of security, compliance and resilience governance controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="32" t="inlineStr">
+        <is>
+          <t>5315-A GOV-02</t>
+        </is>
+      </c>
+      <c r="B1721" s="32" t="inlineStr">
+        <is>
+          <t>Introduction / Compliance</t>
+        </is>
+      </c>
+      <c r="C1721" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to comply with CDT-issued information security and privacy policies and all applicable laws, regulations, rules, and standards governing the state entity.</t>
+        </is>
+      </c>
+      <c r="D1721" s="23" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E1721" s="23" t="inlineStr">
+        <is>
+          <t>Statutory, Regulatory &amp; Contractual Compliance</t>
+        </is>
+      </c>
+      <c r="F1721" s="23" t="inlineStr">
+        <is>
+          <t>CPL-01</t>
+        </is>
+      </c>
+      <c r="G1721" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to facilitate the identification and implementation of relevant statutory, regulatory and contractual controls.</t>
+        </is>
+      </c>
+      <c r="H1721" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1721" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1721" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1721" s="32" t="inlineStr">
+        <is>
+          <t>The requirement to comply with CDT-issued policies and applicable laws/regulations/standards is a specific instance of CPL-01's general mandate to identify and implement relevant statutory, regulatory and contractual controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-01c</t>
+        </is>
+      </c>
+      <c r="B1722" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1722" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement DKIM (DomainKeys Identified Mail) to cryptographically validate email origin and integrity.</t>
+        </is>
+      </c>
+      <c r="D1722" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1722" s="23" t="inlineStr">
+        <is>
+          <t>Domain-Based Message Authentication Reporting and Conformance (DMARC)</t>
+        </is>
+      </c>
+      <c r="F1722" s="23" t="inlineStr">
+        <is>
+          <t>NET-20.4</t>
+        </is>
+      </c>
+      <c r="G1722" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement domain signature verification protections that authenticate incoming email according to the Domain-based Message Authentication Reporting and Conformance (DMARC).</t>
+        </is>
+      </c>
+      <c r="H1722" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1722" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1722" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1722" s="32" t="inlineStr">
+        <is>
+          <t>DKIM is one of the underlying authentication mechanisms DMARC relies on for alignment checks, so the two overlap but DMARC (NET-20.4) is the broader policy-enforcement layer, not DKIM itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-02</t>
+        </is>
+      </c>
+      <c r="B1723" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1723" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to configure SPF records to Hard Fail (reject) rather than Soft Fail (flag) unauthorized senders.</t>
+        </is>
+      </c>
+      <c r="D1723" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1723" s="23" t="inlineStr">
+        <is>
+          <t>Sender Policy Framework (SPF)</t>
+        </is>
+      </c>
+      <c r="F1723" s="23" t="inlineStr">
+        <is>
+          <t>NET-10.3</t>
+        </is>
+      </c>
+      <c r="G1723" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to validate the legitimacy of email communications through configuring a Domain Naming Service (DNS) Sender Policy Framework (SPF) record to specify the IP addresses and/or hostnames that are authorized to send email from the specified domain.</t>
+        </is>
+      </c>
+      <c r="H1723" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1723" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1723" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1723" s="32" t="inlineStr">
+        <is>
+          <t>Adjusting SPF from Soft Fail to Hard Fail is a specific configuration requirement within NET-10.3's broader SPF implementation control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-03</t>
+        </is>
+      </c>
+      <c r="B1724" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1724" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to incorporate vendor-provided threat intelligence into email protection capabilities.</t>
+        </is>
+      </c>
+      <c r="D1724" s="23" t="inlineStr">
+        <is>
+          <t>Threat Management</t>
+        </is>
+      </c>
+      <c r="E1724" s="23" t="inlineStr">
+        <is>
+          <t>Threat Intelligence Feeds</t>
+        </is>
+      </c>
+      <c r="F1724" s="23" t="inlineStr">
+        <is>
+          <t>THR-03</t>
+        </is>
+      </c>
+      <c r="G1724" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to maintain situational awareness of vulnerabilities and evolving threats by leveraging the knowledge of attacker tactics, techniques and procedures to facilitate the implementation of preventative and compensating controls.</t>
+        </is>
+      </c>
+      <c r="H1724" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1724" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1724" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1724" s="32" t="inlineStr">
+        <is>
+          <t>Using vendor-provided threat intelligence to inform email protections is a specific instance of THR-03's mandate to leverage threat intelligence feeds for situational awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-04</t>
+        </is>
+      </c>
+      <c r="B1725" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1725" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to detect email spoofing of both internal and external domains.</t>
+        </is>
+      </c>
+      <c r="D1725" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1725" s="23" t="inlineStr">
+        <is>
+          <t>Domain-Based Message Authentication Reporting and Conformance (DMARC)</t>
+        </is>
+      </c>
+      <c r="F1725" s="23" t="inlineStr">
+        <is>
+          <t>NET-20.4</t>
+        </is>
+      </c>
+      <c r="G1725" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement domain signature verification protections that authenticate incoming email according to the Domain-based Message Authentication Reporting and Conformance (DMARC).</t>
+        </is>
+      </c>
+      <c r="H1725" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1725" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1725" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1725" s="32" t="inlineStr">
+        <is>
+          <t>DMARC is a primary mechanism for detecting/preventing domain spoofing, but this FDE's spoofing-detection requirement is broader than DMARC's specific authentication-and-policy-enforcement mechanism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-06b</t>
+        </is>
+      </c>
+      <c r="B1726" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1726" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to ensure email encryption uses FIPS 140-3 validated cryptographic algorithms and modules.</t>
+        </is>
+      </c>
+      <c r="D1726" s="23" t="inlineStr">
+        <is>
+          <t>Cryptographic Protections</t>
+        </is>
+      </c>
+      <c r="E1726" s="23" t="inlineStr">
+        <is>
+          <t>Use of Cryptographic Controls</t>
+        </is>
+      </c>
+      <c r="F1726" s="23" t="inlineStr">
+        <is>
+          <t>CRY-01</t>
+        </is>
+      </c>
+      <c r="G1726" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to facilitate the implementation of cryptographic protections controls using known public standards and trusted cryptographic technologies.</t>
+        </is>
+      </c>
+      <c r="H1726" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1726" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1726" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1726" s="32" t="inlineStr">
+        <is>
+          <t>Requiring FIPS 140-3 validated cryptographic algorithms/modules for email encryption is a specific instance of CRY-01's general mandate to use approved cryptographic controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-07</t>
+        </is>
+      </c>
+      <c r="B1727" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1727" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to enforce multi-factor authentication for remote access sessions to email.</t>
+        </is>
+      </c>
+      <c r="D1727" s="23" t="inlineStr">
+        <is>
+          <t>Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="E1727" s="23" t="inlineStr">
+        <is>
+          <t>Multi-Factor Authentication (MFA)</t>
+        </is>
+      </c>
+      <c r="F1727" s="23" t="inlineStr">
+        <is>
+          <t>IAC-06</t>
+        </is>
+      </c>
+      <c r="G1727" s="24" t="inlineStr">
+        <is>
+          <t>Automated mechanisms exist to enforce Multi-Factor Authentication (MFA) for:
+(1) Remote network access; 
+(2) Third-party Technology Assets, Applications and/or Services (TAAS); and/ or
+(3) Non-console access to critical TAAS that store, transmit and/or process sensitive and/or regulated data.</t>
+        </is>
+      </c>
+      <c r="H1727" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1727" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1727" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1727" s="32" t="inlineStr">
+        <is>
+          <t>Enforcing MFA for remote access to email is a specific instance of IAC-06's mandate to enforce MFA for remote network access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-10a</t>
+        </is>
+      </c>
+      <c r="B1728" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1728" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to disable external email auto-forwarding rules by default.</t>
+        </is>
+      </c>
+      <c r="D1728" s="23" t="n"/>
+      <c r="E1728" s="23" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="F1728" s="23" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="G1728" s="24" t="n"/>
+      <c r="H1728" s="32" t="n"/>
+      <c r="I1728" s="33" t="inlineStr">
+        <is>
+          <t>NO RELATIONSHIP</t>
+        </is>
+      </c>
+      <c r="J1728" s="33" t="n"/>
+      <c r="K1728" s="32" t="inlineStr">
+        <is>
+          <t>No SCF v2026.2 control found with a genuine, substantive match to this SIMM 5315-A provision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-10c</t>
+        </is>
+      </c>
+      <c r="B1729" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1729" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to periodically review approved auto-forwarding exceptions and spot-check forwarded messages for authorized recipients and indicators of compromise.</t>
+        </is>
+      </c>
+      <c r="D1729" s="23" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="E1729" s="23" t="inlineStr">
+        <is>
+          <t>Periodic Audits</t>
+        </is>
+      </c>
+      <c r="F1729" s="23" t="inlineStr">
+        <is>
+          <t>CPL-02.2</t>
+        </is>
+      </c>
+      <c r="G1729" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to conduct periodic audits of security, compliance and resilience controls to evaluate conformity with the organization's documented policies, standards and procedures.</t>
+        </is>
+      </c>
+      <c r="H1729" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1729" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1729" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1729" s="32" t="inlineStr">
+        <is>
+          <t>Periodically reviewing and spot-checking auto-forwarding exceptions is a specific case of CPL-02.2's broader periodic-audit mandate for conformity with policies, though CPL-02.2 is not specific to forwarding exceptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-10d</t>
+        </is>
+      </c>
+      <c r="B1730" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1730" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to apply DLP to outbound email where an auto-forwarding exception has been granted.</t>
+        </is>
+      </c>
+      <c r="D1730" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1730" s="23" t="inlineStr">
+        <is>
+          <t>Data Loss Prevention (DLP)</t>
+        </is>
+      </c>
+      <c r="F1730" s="23" t="inlineStr">
+        <is>
+          <t>NET-17</t>
+        </is>
+      </c>
+      <c r="G1730" s="24" t="inlineStr">
+        <is>
+          <t>Automated mechanisms exist to implement Data Loss Prevention (DLP) to protect sensitive information as it is stored, transmitted and processed.</t>
+        </is>
+      </c>
+      <c r="H1730" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1730" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1730" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1730" s="32" t="inlineStr">
+        <is>
+          <t>Applying DLP to outbound email where a forwarding exception exists is a specific instance of NET-17's general DLP mandate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-11</t>
+        </is>
+      </c>
+      <c r="B1731" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1731" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to add a notification banner to inbound email originating from external domains.</t>
+        </is>
+      </c>
+      <c r="D1731" s="23" t="n"/>
+      <c r="E1731" s="23" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="F1731" s="23" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="G1731" s="24" t="n"/>
+      <c r="H1731" s="32" t="n"/>
+      <c r="I1731" s="33" t="inlineStr">
+        <is>
+          <t>NO RELATIONSHIP</t>
+        </is>
+      </c>
+      <c r="J1731" s="33" t="n"/>
+      <c r="K1731" s="32" t="inlineStr">
+        <is>
+          <t>No SCF v2026.2 control found with a genuine, substantive match to this SIMM 5315-A provision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-13</t>
+        </is>
+      </c>
+      <c r="B1732" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1732" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict link-sharing permissions in email using a zero-trust, Role-Based Access Control (RBAC) framework.</t>
+        </is>
+      </c>
+      <c r="D1732" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1732" s="23" t="inlineStr">
+        <is>
+          <t>Zero Trust Architecture (ZTA)</t>
+        </is>
+      </c>
+      <c r="F1732" s="23" t="inlineStr">
+        <is>
+          <t>NET-01.1</t>
+        </is>
+      </c>
+      <c r="G1732" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to treat all users and devices as potential threats and prevent access to data and resources until the users can be properly authenticated and their access authorized.</t>
+        </is>
+      </c>
+      <c r="H1732" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1732" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1732" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1732" s="32" t="inlineStr">
+        <is>
+          <t>Restricting link-sharing via a zero-trust framework overlaps with NET-01.1's zero trust architecture principle of not implicitly trusting access, though NET-01.1 is a broad architectural control rather than an email-link-specific one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="32" t="inlineStr">
+        <is>
+          <t>5315-A PROT-13</t>
+        </is>
+      </c>
+      <c r="B1733" s="32" t="inlineStr">
+        <is>
+          <t>Protection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1733" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict link-sharing permissions in email using a zero-trust, Role-Based Access Control (RBAC) framework.</t>
+        </is>
+      </c>
+      <c r="D1733" s="23" t="inlineStr">
+        <is>
+          <t>Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="E1733" s="23" t="inlineStr">
+        <is>
+          <t>Role-Based Access Control (RBAC)</t>
+        </is>
+      </c>
+      <c r="F1733" s="23" t="inlineStr">
+        <is>
+          <t>IAC-08</t>
+        </is>
+      </c>
+      <c r="G1733" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to enforce Role-Based Access Control (RBAC) for Technology Assets, Applications, Services and/or Data (TAASD) to restrict access to individuals assigned specific roles with legitimate business needs.</t>
+        </is>
+      </c>
+      <c r="H1733" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1733" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1733" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1733" s="32" t="inlineStr">
+        <is>
+          <t>Role-Based Access Control for link-sharing permissions overlaps with IAC-08's general RBAC mandate, though IAC-08 is scoped to Technology Assets/Applications/Services/Data broadly rather than email link-sharing specifically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="32" t="inlineStr">
+        <is>
+          <t>5315-A DET-00</t>
+        </is>
+      </c>
+      <c r="B1734" s="32" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1734" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to correlate detection alerts into events and prioritize incident response based on confidence level, severity, and risk.</t>
+        </is>
+      </c>
+      <c r="D1734" s="23" t="inlineStr">
+        <is>
+          <t>Continuous Monitoring</t>
+        </is>
+      </c>
+      <c r="E1734" s="23" t="inlineStr">
+        <is>
+          <t>Correlate Monitoring Information</t>
+        </is>
+      </c>
+      <c r="F1734" s="23" t="inlineStr">
+        <is>
+          <t>MON-02.1</t>
+        </is>
+      </c>
+      <c r="G1734" s="24" t="inlineStr">
+        <is>
+          <t>Automated mechanisms exist to correlate both technical and non-technical information from across the enterprise by a Security Incident Event Manager (SIEM) or similar automated tool, to enhance organization-wide situational awareness.</t>
+        </is>
+      </c>
+      <c r="H1734" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1734" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1734" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1734" s="32" t="inlineStr">
+        <is>
+          <t>Correlating detection alerts into events and prioritizing response by confidence/severity/risk is a specific instance of MON-02.1's mandate to correlate monitoring information via a SIEM or similar tool for situational awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="32" t="inlineStr">
+        <is>
+          <t>5315-A DET-01</t>
+        </is>
+      </c>
+      <c r="B1735" s="32" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1735" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to screen inbound email for spam, phishing, and malicious intent using heuristics and machine learning, quarantining likely malicious or phishing emails.</t>
+        </is>
+      </c>
+      <c r="D1735" s="23" t="inlineStr">
+        <is>
+          <t>Endpoint Security</t>
+        </is>
+      </c>
+      <c r="E1735" s="23" t="inlineStr">
+        <is>
+          <t>Phishing &amp; Spam Protection</t>
+        </is>
+      </c>
+      <c r="F1735" s="23" t="inlineStr">
+        <is>
+          <t>END-08</t>
+        </is>
+      </c>
+      <c r="G1735" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to utilize anti-phishing and spam protection technologies to detect and take action on unsolicited messages transported by electronic mail.</t>
+        </is>
+      </c>
+      <c r="H1735" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1735" s="32" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1735" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1735" s="32" t="inlineStr">
+        <is>
+          <t>Both require screening email for spam/phishing/malicious intent using heuristics and intelligent techniques and taking action (quarantine); scope is essentially identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="32" t="inlineStr">
+        <is>
+          <t>5315-A DET-02</t>
+        </is>
+      </c>
+      <c r="B1736" s="32" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1736" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to screen email attachments using malware analysis, sandboxing, and machine learning to block malicious attachments, including zero-day threats, prior to delivery.</t>
+        </is>
+      </c>
+      <c r="D1736" s="23" t="inlineStr">
+        <is>
+          <t>Endpoint Security</t>
+        </is>
+      </c>
+      <c r="E1736" s="23" t="inlineStr">
+        <is>
+          <t>Malicious Code Protection (Anti-Malware)</t>
+        </is>
+      </c>
+      <c r="F1736" s="23" t="inlineStr">
+        <is>
+          <t>END-04</t>
+        </is>
+      </c>
+      <c r="G1736" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to utilize antimalware technologies to detect and eradicate malicious code.</t>
+        </is>
+      </c>
+      <c r="H1736" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1736" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1736" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1736" s="32" t="inlineStr">
+        <is>
+          <t>END-04's general anti-malware technology mandate overlaps with attachment malware screening, though it is not specific to email attachments or sandboxing/zero-day detection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="32" t="inlineStr">
+        <is>
+          <t>5315-A DET-03</t>
+        </is>
+      </c>
+      <c r="B1737" s="32" t="inlineStr">
+        <is>
+          <t>Detection Capabilities</t>
+        </is>
+      </c>
+      <c r="C1737" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to screen links in email messages at time-of-click, evaluating target site reputation and content, to block or warn users of unsafe links.</t>
+        </is>
+      </c>
+      <c r="D1737" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1737" s="23" t="inlineStr">
+        <is>
+          <t>DNS &amp; Content Filtering</t>
+        </is>
+      </c>
+      <c r="F1737" s="23" t="inlineStr">
+        <is>
+          <t>NET-18</t>
+        </is>
+      </c>
+      <c r="G1737" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to force Internet-bound network traffic through a proxy device (e.g., Policy Enforcement Point (PEP)) for URL content filtering and DNS filtering to limit a user's ability to connect to dangerous or prohibited Internet sites.</t>
+        </is>
+      </c>
+      <c r="H1737" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1737" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1737" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1737" s="32" t="inlineStr">
+        <is>
+          <t>Time-of-click URL reputation screening overlaps with NET-18's URL content filtering/DNS filtering mandate, though NET-18 is framed around proxying general Internet-bound traffic rather than email-embedded links specifically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-01</t>
+        </is>
+      </c>
+      <c r="B1738" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1738" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to forward logs of security-related email actions (malicious/spam/phishing detections, attachment detections, URL clicks, DLP hits) to a designated SIEM system.</t>
+        </is>
+      </c>
+      <c r="D1738" s="23" t="inlineStr">
+        <is>
+          <t>Continuous Monitoring</t>
+        </is>
+      </c>
+      <c r="E1738" s="23" t="inlineStr">
+        <is>
+          <t>Centralized Collection of Security Event Logs</t>
+        </is>
+      </c>
+      <c r="F1738" s="23" t="inlineStr">
+        <is>
+          <t>MON-02</t>
+        </is>
+      </c>
+      <c r="G1738" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to utilize a Security Incident Event Manager (SIEM), or similar automated tool, to support the centralized collection of security-related event logs.</t>
+        </is>
+      </c>
+      <c r="H1738" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1738" s="32" t="inlineStr">
+        <is>
+          <t>EQUAL</t>
+        </is>
+      </c>
+      <c r="J1738" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1738" s="32" t="inlineStr">
+        <is>
+          <t>Both require forwarding security-related logs to a centralized SIEM (or similar tool); scope is essentially identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-02</t>
+        </is>
+      </c>
+      <c r="B1739" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1739" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to transmit pertinent cyber threat information, consistent with NIST SP 800-150, to the California Department of Technology.</t>
+        </is>
+      </c>
+      <c r="D1739" s="23" t="inlineStr">
+        <is>
+          <t>Threat Management</t>
+        </is>
+      </c>
+      <c r="E1739" s="23" t="inlineStr">
+        <is>
+          <t>Threat Intelligence Program</t>
+        </is>
+      </c>
+      <c r="F1739" s="23" t="inlineStr">
+        <is>
+          <t>THR-01</t>
+        </is>
+      </c>
+      <c r="G1739" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement a threat intelligence program that includes a cross-organization information-sharing capability that can influence the development of the system and security architectures, selection of security solutions, monitoring, threat hunting, response and recovery activities.</t>
+        </is>
+      </c>
+      <c r="H1739" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1739" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1739" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1739" s="32" t="inlineStr">
+        <is>
+          <t>Passing threat information per NIST SP 800-150 to CDT overlaps with THR-01's cross-organization information-sharing capability, though THR-01 is a broader internal threat-intel program rather than this specific external reporting obligation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-03</t>
+        </is>
+      </c>
+      <c r="B1740" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1740" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provide a reporting environment supporting deep investigation, message tracing, summarization, and URL link-click tracking.</t>
+        </is>
+      </c>
+      <c r="D1740" s="23" t="inlineStr">
+        <is>
+          <t>Continuous Monitoring</t>
+        </is>
+      </c>
+      <c r="E1740" s="23" t="inlineStr">
+        <is>
+          <t>Correlate Monitoring Information</t>
+        </is>
+      </c>
+      <c r="F1740" s="23" t="inlineStr">
+        <is>
+          <t>MON-02.1</t>
+        </is>
+      </c>
+      <c r="G1740" s="24" t="inlineStr">
+        <is>
+          <t>Automated mechanisms exist to correlate both technical and non-technical information from across the enterprise by a Security Incident Event Manager (SIEM) or similar automated tool, to enhance organization-wide situational awareness.</t>
+        </is>
+      </c>
+      <c r="H1740" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1740" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1740" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1740" s="32" t="inlineStr">
+        <is>
+          <t>A rich reporting environment for message tracing/summarization/link-click tracking overlaps with MON-02.1's correlation of monitoring information for situational awareness, though MON-02.1 is not specific to email message tracing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-04</t>
+        </is>
+      </c>
+      <c r="B1741" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1741" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to establish and maintain a dedicated email address for the State Security Operations Center (SOC) to notify impacted entities of anomalies and suspected or confirmed incidents.</t>
+        </is>
+      </c>
+      <c r="D1741" s="23" t="inlineStr">
+        <is>
+          <t>Incident Response</t>
+        </is>
+      </c>
+      <c r="E1741" s="23" t="inlineStr">
+        <is>
+          <t>Incident Stakeholder Reporting</t>
+        </is>
+      </c>
+      <c r="F1741" s="23" t="inlineStr">
+        <is>
+          <t>IRO-10</t>
+        </is>
+      </c>
+      <c r="G1741" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to timely-report incidents to applicable:
+(1) Internal stakeholders; 
+(2) Affected clients &amp; third-parties; and
+(3) Regulatory authorities.</t>
+        </is>
+      </c>
+      <c r="H1741" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1741" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1741" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1741" s="32" t="inlineStr">
+        <is>
+          <t>Establishing a dedicated SOC notification address to notify impacted entities of incidents is a specific instance of IRO-10's mandate to timely-report incidents to internal stakeholders and affected clients/third-parties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-05</t>
+        </is>
+      </c>
+      <c r="B1742" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1742" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to ensure SOC notification email addresses follow the standardized naming convention [Entity Acronym].SOC.Notifications@[domain].ca.gov.</t>
+        </is>
+      </c>
+      <c r="D1742" s="23" t="inlineStr">
+        <is>
+          <t>Incident Response</t>
+        </is>
+      </c>
+      <c r="E1742" s="23" t="inlineStr">
+        <is>
+          <t>Incident Stakeholder Reporting</t>
+        </is>
+      </c>
+      <c r="F1742" s="23" t="inlineStr">
+        <is>
+          <t>IRO-10</t>
+        </is>
+      </c>
+      <c r="G1742" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to timely-report incidents to applicable:
+(1) Internal stakeholders; 
+(2) Affected clients &amp; third-parties; and
+(3) Regulatory authorities.</t>
+        </is>
+      </c>
+      <c r="H1742" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1742" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1742" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1742" s="32" t="inlineStr">
+        <is>
+          <t>The specific naming-convention requirement for the SOC address is a narrow administrative detail of the broader stakeholder-reporting mechanism IRO-10 covers; no SCF control addresses naming conventions specifically, so this is only a nominal link to the parent reporting control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-06</t>
+        </is>
+      </c>
+      <c r="B1743" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1743" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to ensure individuals required to acknowledge a SOC notification within two hours are included as contacts on the group email address.</t>
+        </is>
+      </c>
+      <c r="D1743" s="23" t="inlineStr">
+        <is>
+          <t>Incident Response</t>
+        </is>
+      </c>
+      <c r="E1743" s="23" t="inlineStr">
+        <is>
+          <t>Incident Stakeholder Reporting</t>
+        </is>
+      </c>
+      <c r="F1743" s="23" t="inlineStr">
+        <is>
+          <t>IRO-10</t>
+        </is>
+      </c>
+      <c r="G1743" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to timely-report incidents to applicable:
+(1) Internal stakeholders; 
+(2) Affected clients &amp; third-parties; and
+(3) Regulatory authorities.</t>
+        </is>
+      </c>
+      <c r="H1743" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1743" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1743" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1743" s="32" t="inlineStr">
+        <is>
+          <t>Ensuring the right individuals are subscribed to acknowledge SOC notifications within 2 hours supports the stakeholder-reporting mechanism in IRO-10, but the specific staffing/ack-time requirement is not itself addressed by any SCF control -- only a nominal link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="32" t="inlineStr">
+        <is>
+          <t>5315-A INV-07</t>
+        </is>
+      </c>
+      <c r="B1744" s="32" t="inlineStr">
+        <is>
+          <t>Investigative Support Capabilities</t>
+        </is>
+      </c>
+      <c r="C1744" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provide timely supplemental investigative findings to the SOC.</t>
+        </is>
+      </c>
+      <c r="D1744" s="23" t="inlineStr">
+        <is>
+          <t>Incident Response</t>
+        </is>
+      </c>
+      <c r="E1744" s="23" t="inlineStr">
+        <is>
+          <t>Situational Awareness For Incidents</t>
+        </is>
+      </c>
+      <c r="F1744" s="23" t="inlineStr">
+        <is>
+          <t>IRO-09</t>
+        </is>
+      </c>
+      <c r="G1744" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to document, monitor and report the status of cybersecurity and data protection incidents to internal stakeholders all the way through the resolution of the incident.</t>
+        </is>
+      </c>
+      <c r="H1744" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1744" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1744" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1744" s="32" t="inlineStr">
+        <is>
+          <t>Providing timely supplemental investigative findings to the SOC overlaps with IRO-09's mandate to document, monitor and report incident status to stakeholders through resolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="32" t="inlineStr">
+        <is>
+          <t>5315-A CON-01</t>
+        </is>
+      </c>
+      <c r="B1745" s="32" t="inlineStr">
+        <is>
+          <t>Containment Capabilities</t>
+        </is>
+      </c>
+      <c r="C1745" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to manually or automatically quarantine and/or remove emails deemed malicious or dangerous in a timely manner.</t>
+        </is>
+      </c>
+      <c r="D1745" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1745" s="23" t="inlineStr">
+        <is>
+          <t>Email Content Protections</t>
+        </is>
+      </c>
+      <c r="F1745" s="23" t="inlineStr">
+        <is>
+          <t>NET-20</t>
+        </is>
+      </c>
+      <c r="G1745" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement an email filtering security service to detect malicious attachments in emails and prevent users from accessing them.</t>
+        </is>
+      </c>
+      <c r="H1745" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1745" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1745" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1745" s="32" t="inlineStr">
+        <is>
+          <t>Quarantining/removing malicious or dangerous email closely overlaps with NET-20's email filtering service that detects malicious content and prevents user access to it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="32" t="inlineStr">
+        <is>
+          <t>5315-A CON-01</t>
+        </is>
+      </c>
+      <c r="B1746" s="32" t="inlineStr">
+        <is>
+          <t>Containment Capabilities</t>
+        </is>
+      </c>
+      <c r="C1746" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to manually or automatically quarantine and/or remove emails deemed malicious or dangerous in a timely manner.</t>
+        </is>
+      </c>
+      <c r="D1746" s="23" t="inlineStr">
+        <is>
+          <t>Endpoint Security</t>
+        </is>
+      </c>
+      <c r="E1746" s="23" t="inlineStr">
+        <is>
+          <t>Phishing &amp; Spam Protection</t>
+        </is>
+      </c>
+      <c r="F1746" s="23" t="inlineStr">
+        <is>
+          <t>END-08</t>
+        </is>
+      </c>
+      <c r="G1746" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to utilize anti-phishing and spam protection technologies to detect and take action on unsolicited messages transported by electronic mail.</t>
+        </is>
+      </c>
+      <c r="H1746" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1746" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1746" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1746" s="32" t="inlineStr">
+        <is>
+          <t>END-08's anti-phishing/spam technologies that 'detect and take action' on unsolicited/malicious messages overlaps with quarantine/removal containment, though END-08 is framed around phishing/spam rather than malicious email broadly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="32" t="inlineStr">
+        <is>
+          <t>5315-A REM-01</t>
+        </is>
+      </c>
+      <c r="B1747" s="32" t="inlineStr">
+        <is>
+          <t>Remediation Capabilities</t>
+        </is>
+      </c>
+      <c r="C1747" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement custom filtering of incoming email to screen for previously detected malicious emails.</t>
+        </is>
+      </c>
+      <c r="D1747" s="23" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="E1747" s="23" t="inlineStr">
+        <is>
+          <t>Email Content Protections</t>
+        </is>
+      </c>
+      <c r="F1747" s="23" t="inlineStr">
+        <is>
+          <t>NET-20</t>
+        </is>
+      </c>
+      <c r="G1747" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to implement an email filtering security service to detect malicious attachments in emails and prevent users from accessing them.</t>
+        </is>
+      </c>
+      <c r="H1747" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1747" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1747" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1747" s="32" t="inlineStr">
+        <is>
+          <t>Custom filtering of incoming email to screen previously detected malicious emails overlaps with NET-20's email filtering service, though NET-20 is framed around attachment detection rather than custom rule-based re-filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="32" t="inlineStr">
+        <is>
+          <t>5315-A OPT-01</t>
+        </is>
+      </c>
+      <c r="B1748" s="32" t="inlineStr">
+        <is>
+          <t>Above-Minimum / Optional Capabilities</t>
+        </is>
+      </c>
+      <c r="C1748" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to provision and de-provision individual and group user access for remote access to email.</t>
+        </is>
+      </c>
+      <c r="D1748" s="23" t="inlineStr">
+        <is>
+          <t>Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="E1748" s="23" t="inlineStr">
+        <is>
+          <t>User Provisioning &amp; De-Provisioning</t>
+        </is>
+      </c>
+      <c r="F1748" s="23" t="inlineStr">
+        <is>
+          <t>IAC-07</t>
+        </is>
+      </c>
+      <c r="G1748" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to utilize a formal user registration and de-registration process that governs the assignment of access rights.</t>
+        </is>
+      </c>
+      <c r="H1748" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1748" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1748" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1748" s="32" t="inlineStr">
+        <is>
+          <t>Provisioning/de-provisioning individual and group remote-access email users is a specific instance of IAC-07's mandate for a formal user registration/de-registration process governing access rights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="32" t="inlineStr">
+        <is>
+          <t>5315-A OPT-02</t>
+        </is>
+      </c>
+      <c r="B1749" s="32" t="inlineStr">
+        <is>
+          <t>Above-Minimum / Optional Capabilities</t>
+        </is>
+      </c>
+      <c r="C1749" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to restrict who may send to group/distribution email lists, preventing external entities from using an entity's internal distribution lists.</t>
+        </is>
+      </c>
+      <c r="D1749" s="23" t="inlineStr">
+        <is>
+          <t>Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="E1749" s="23" t="inlineStr">
+        <is>
+          <t>Role-Based Access Control (RBAC)</t>
+        </is>
+      </c>
+      <c r="F1749" s="23" t="inlineStr">
+        <is>
+          <t>IAC-08</t>
+        </is>
+      </c>
+      <c r="G1749" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to enforce Role-Based Access Control (RBAC) for Technology Assets, Applications, Services and/or Data (TAASD) to restrict access to individuals assigned specific roles with legitimate business needs.</t>
+        </is>
+      </c>
+      <c r="H1749" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1749" s="32" t="inlineStr">
+        <is>
+          <t>INTERSECTS WITH</t>
+        </is>
+      </c>
+      <c r="J1749" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1749" s="32" t="inlineStr">
+        <is>
+          <t>Role-based restriction of who may send to a distribution list overlaps with IAC-08's general RBAC mandate, though IAC-08 is not specific to email distribution lists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="32" t="inlineStr">
+        <is>
+          <t>5315-A OPT-03</t>
+        </is>
+      </c>
+      <c r="B1750" s="32" t="inlineStr">
+        <is>
+          <t>Above-Minimum / Optional Capabilities</t>
+        </is>
+      </c>
+      <c r="C1750" s="32" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to support state entity-specific acceptable use policies and standards for email.</t>
+        </is>
+      </c>
+      <c r="D1750" s="23" t="inlineStr">
+        <is>
+          <t>Human Resources Security</t>
+        </is>
+      </c>
+      <c r="E1750" s="23" t="inlineStr">
+        <is>
+          <t>Rules of Behavior</t>
+        </is>
+      </c>
+      <c r="F1750" s="23" t="inlineStr">
+        <is>
+          <t>HRS-05.1</t>
+        </is>
+      </c>
+      <c r="G1750" s="24" t="inlineStr">
+        <is>
+          <t>Mechanisms exist to define acceptable and unacceptable rules of behavior for the use of technologies, including consequences for unacceptable behavior.</t>
+        </is>
+      </c>
+      <c r="H1750" s="32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="I1750" s="32" t="inlineStr">
+        <is>
+          <t>SUBSET OF</t>
+        </is>
+      </c>
+      <c r="J1750" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1750" s="32" t="inlineStr">
+        <is>
+          <t>Supporting entity-specific acceptable use policies/standards for email is a specific instance of HRS-05.1's mandate to define acceptable/unacceptable rules of behavior for use of technologies.</t>
         </is>
       </c>
     </row>

</xml_diff>